<commit_message>
Rename Cooling Demand terminology to Cooling Potential
Aligns column names, translations (EN/FR/PT), both data dictionaries, and
the visualization platform with SEforALL's updated naming (CDI/PHCDI/FCDI
-> CPI/PHCPI/FCPI). Mirrors the same rename applied in AgCAP_MOZ, adapted
to this repo's numbered notebook pipeline and irrigation module.

Re-ran 3_core_analysis_engine.ipynb -> 4_Contextuals_Extraction.ipynb ->
5_Irrigation_Extraction.ipynb -> 6_SDI_Integration.ipynb to regenerate
exported data with the new column names.
</commit_message>
<xml_diff>
--- a/docs/settlements_data_dictionary_MOZ.xlsx
+++ b/docs/settlements_data_dictionary_MOZ.xlsx
@@ -1142,7 +1142,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Agricultural Cooling Demand</t>
+          <t>Agricultural Cooling Potential</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1152,75 +1152,75 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Composite indicator of market accessibility to export markets. Weighted average of nearby population, travel times to capital city, nearest cities, airports,ports, railway stations (0=lowest, 1=highest)</t>
+          <t>Composite indicator of farming activity. Weighted average of nearby population, travel times to capital city, nearest cities, airports,ports, railway stations (0=lowest, 1=highest)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Agricultural Cooling Demand</t>
+          <t>Agricultural Cooling Potential</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Ag Cooling Demand Export Market</t>
+          <t>Ag Cooling Potential Export Market</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Composite indicator of cooling demand for fish products destined for export markets (0=lowest, 1=highest)</t>
+          <t>Composite indicator of cooling potential for agricultural products destined for export markets (0=lowest, 1=highest)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Agricultural Cooling Demand</t>
+          <t>Agricultural Cooling Potential</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ag Cooling Demand National Market</t>
+          <t>Ag Cooling Potential National Market</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Composite indicator of cooling demand for fish products destined for national distribution (0=lowest, 1=highest)</t>
+          <t>Composite indicator of cooling potential for agricultural products destined for national distribution (0=lowest, 1=highest)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Agricultural Cooling Demand</t>
+          <t>Agricultural Cooling Potential</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ag Cooling Demand Fresh Markets</t>
+          <t>Ag Cooling Potential Fresh Markets</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Composite indicator of cooling demand for fish products destined for local fresh markets (0=lowest, 1=highest)</t>
+          <t>Composite indicator of cooling potential for agricultural products destined for local fresh markets (0=lowest, 1=highest)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Agricultural Cooling Demand</t>
+          <t>Agricultural Cooling Potential</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ag Cooling Demand ALL Markets</t>
+          <t>Ag Cooling Potential ALL Markets</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Composite indicator of cooling demand for fish products across all destination markets (0=lowest, 1=highest)</t>
+          <t>Composite indicator of cooling potential for agricultural products across all destination markets (0=lowest, 1=highest)</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Fishing Cooling Demand</t>
+          <t>Fishing Cooling Potential</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1431,7 +1431,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Fishing Cooling Demand</t>
+          <t>Fishing Cooling Potential</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1448,7 +1448,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Fishing Cooling Demand</t>
+          <t>Fishing Cooling Potential</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Fishing Cooling Demand</t>
+          <t>Fishing Cooling Potential</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1482,12 +1482,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Fishing Cooling Demand</t>
+          <t>Fishing Cooling Potential</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Fish Cooling Demand Export Market</t>
+          <t>Fish Cooling Potential Export Market</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1499,12 +1499,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Fishing Cooling Demand</t>
+          <t>Fishing Cooling Potential</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Fish Cooling Demand National Market</t>
+          <t>Fish Cooling Potential National Market</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1516,12 +1516,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Fishing Cooling Demand</t>
+          <t>Fishing Cooling Potential</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Fish Cooling Demand Fresh Markets</t>
+          <t>Fish Cooling Potential Fresh Markets</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1533,12 +1533,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Fishing Cooling Demand</t>
+          <t>Fishing Cooling Potential</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Fish Cooling Demand ALL Markets</t>
+          <t>Fish Cooling Potential ALL Markets</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2278,7 +2278,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração Agrícola</t>
+          <t>Potencial de Refrigeração Agrícola</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2295,68 +2295,68 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração Agrícola</t>
+          <t>Potencial de Refrigeração Agrícola</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração Agrícola - Mercado de Exportação</t>
+          <t>Potencial de Refrigeração Agrícola - Mercado de Exportação</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Indicador composto de demanda de refrigeração para produtos agrícolas destinados a mercados de exportação (0=mais baixo, 1=mais alto)</t>
+          <t>Indicador composto de potencial de refrigeração para produtos agrícolas destinados a mercados de exportação (0=mais baixo, 1=mais alto)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração Agrícola</t>
+          <t>Potencial de Refrigeração Agrícola</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração Agrícola - Mercado Nacional</t>
+          <t>Potencial de Refrigeração Agrícola - Mercado Nacional</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Indicador composto de demanda de refrigeração para produtos agrícolas destinados à distribuição nacional (0=mais baixo, 1=mais alto)</t>
+          <t>Indicador composto de potencial de refrigeração para produtos agrícolas destinados à distribuição nacional (0=mais baixo, 1=mais alto)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração Agrícola</t>
+          <t>Potencial de Refrigeração Agrícola</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração Agrícola - Mercados de Produtos Frescos</t>
+          <t>Potencial de Refrigeração Agrícola - Mercados de Produtos Frescos</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Indicador composto de demanda de refrigeração para produtos agrícolas destinados a mercados frescos locais (0=mais baixo, 1=mais alto)</t>
+          <t>Indicador composto de potencial de refrigeração para produtos agrícolas destinados a mercados frescos locais (0=mais baixo, 1=mais alto)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração Agrícola</t>
+          <t>Potencial de Refrigeração Agrícola</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração Agrícola - TODOS os Mercados</t>
+          <t>Potencial de Refrigeração Agrícola - TODOS os Mercados</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Indicador composto de demanda de refrigeração para produtos agrícolas em todos os mercados de destino (0=mais baixo, 1=mais alto)</t>
+          <t>Indicador composto de potencial de refrigeração para produtos agrícolas em todos os mercados de destino (0=mais baixo, 1=mais alto)</t>
         </is>
       </c>
     </row>
@@ -2550,7 +2550,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração na Pesca</t>
+          <t>Potencial de Refrigeração na Pesca</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração na Pesca</t>
+          <t>Potencial de Refrigeração na Pesca</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2584,7 +2584,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração na Pesca</t>
+          <t>Potencial de Refrigeração na Pesca</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2601,7 +2601,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração na Pesca</t>
+          <t>Potencial de Refrigeração na Pesca</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2618,68 +2618,68 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração na Pesca</t>
+          <t>Potencial de Refrigeração na Pesca</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração de Pescado - Mercado de Exportação</t>
+          <t>Potencial de Refrigeração de Pescado - Mercado de Exportação</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Indicador composto de demanda de refrigeração/fabricação de gelo para produtos de pesca destinados a mercados de exportação (0=mais baixo, 1=mais alto)</t>
+          <t>Indicador composto de potencial de refrigeração/fabricação de gelo para produtos de pesca destinados a mercados de exportação (0=mais baixo, 1=mais alto)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração na Pesca</t>
+          <t>Potencial de Refrigeração na Pesca</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração de Pescado - Mercado Nacional</t>
+          <t>Potencial de Refrigeração de Pescado - Mercado Nacional</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Indicador composto de demanda de refrigeração/fabricação de gelo para produtos de pesca destinados à distribuição nacional (0=mais baixo, 1=mais alto)</t>
+          <t>Indicador composto de potencial de refrigeração/fabricação de gelo para produtos de pesca destinados à distribuição nacional (0=mais baixo, 1=mais alto)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração na Pesca</t>
+          <t>Potencial de Refrigeração na Pesca</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração de Pescado - Mercados Frescos</t>
+          <t>Potencial de Refrigeração de Pescado - Mercados Frescos</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Indicador composto de demanda de refrigeração/fabricação de gelo para produtos de pesca destinados a mercados frescos locais (0=mais baixo, 1=mais alto)</t>
+          <t>Indicador composto de potencial de refrigeração/fabricação de gelo para produtos de pesca destinados a mercados frescos locais (0=mais baixo, 1=mais alto)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração na Pesca</t>
+          <t>Potencial de Refrigeração na Pesca</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Demanda de Refrigeração de Pescado - TODOS os Mercados</t>
+          <t>Potencial de Refrigeração de Pescado - TODOS os Mercados</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Indicador composto de demanda de refrigeração/fabricação de gelo para produtos de pesca em todos os mercados de destino (0=mais baixo, 1=mais alto)</t>
+          <t>Indicador composto de potencial de refrigeração/fabricação de gelo para produtos de pesca em todos os mercados de destino (0=mais baixo, 1=mais alto)</t>
         </is>
       </c>
     </row>

</xml_diff>